<commit_message>
Notebook de mise à jour du classeur (données, statistiques, prévision)
</commit_message>
<xml_diff>
--- a/excel/Pharma_Analyse.xlsx
+++ b/excel/Pharma_Analyse.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ventes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Calendrier" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conseils" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prévision" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Questions" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Médicaments" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Méthode" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistiques" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="État des données" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Données" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Synthèse" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ventes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Calendrier" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Conseils" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Prévision" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Questions" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Médicaments" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Méthode" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Statistiques" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="État des données" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Données" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="DateMin">MIN(Données!$A$2:$A$2107)</definedName>
@@ -28,12 +28,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="\+0%;\-0%;0%"/>
     <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="+0.0;-0.0"/>
+    <numFmt numFmtId="169" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="37">
     <font>
@@ -1702,6 +1703,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1" s="76">
       <c r="B4" s="1" t="inlineStr">
         <is>
@@ -1761,6 +1763,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="24" customHeight="1" s="76">
       <c r="A7" s="11" t="inlineStr">
         <is>
@@ -1804,6 +1807,7 @@
       <c r="G9" s="71" t="n"/>
       <c r="H9" s="72" t="n"/>
     </row>
+    <row r="10"/>
     <row r="11" ht="24" customHeight="1" s="76">
       <c r="A11" s="11" t="inlineStr">
         <is>
@@ -1841,6 +1845,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15" ht="24" customHeight="1" s="76">
       <c r="A15" s="11" t="inlineStr">
         <is>
@@ -2250,6 +2255,7 @@
         </is>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="24" customHeight="1" s="76">
       <c r="B27" s="11" t="inlineStr">
         <is>
@@ -2293,6 +2299,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32" ht="24" customHeight="1" s="76">
       <c r="A32" s="11" t="inlineStr">
         <is>
@@ -2567,6 +2574,7 @@
         </is>
       </c>
     </row>
+    <row r="44"/>
     <row r="45" ht="24" customHeight="1" s="76">
       <c r="A45" s="11" t="inlineStr">
         <is>
@@ -2808,7 +2816,7 @@
       </c>
       <c r="D56" s="70" t="inlineStr">
         <is>
-          <t>Testé sur 21 mois ; non pour l'asthme et l'ibuprofène. Voir l'onglet Prévision.</t>
+          <t>Testé sur 21 mois. Voir l'onglet Prévision.</t>
         </is>
       </c>
       <c r="E56" s="71" t="n"/>
@@ -2816,6 +2824,8 @@
       <c r="G56" s="71" t="n"/>
       <c r="H56" s="72" t="n"/>
     </row>
+    <row r="57"/>
+    <row r="58"/>
     <row r="59" ht="24" customHeight="1" s="76">
       <c r="A59" s="11" t="inlineStr">
         <is>
@@ -2991,17 +3001,17 @@
           <t>Prévision ▶</t>
         </is>
       </c>
-      <c r="B69" s="121" t="n"/>
+      <c r="B69" s="139" t="n"/>
       <c r="C69" s="122" t="inlineStr">
         <is>
-          <t>Peut-on prévoir le mois suivant ? Le test, et la prévision d'octobre 2019</t>
-        </is>
-      </c>
-      <c r="D69" s="121" t="n"/>
-      <c r="E69" s="121" t="n"/>
-      <c r="F69" s="121" t="n"/>
-      <c r="G69" s="121" t="n"/>
-      <c r="H69" s="121" t="n"/>
+          <t>Peut-on prévoir le mois suivant ? Le test, et la prévision 10/2019</t>
+        </is>
+      </c>
+      <c r="D69" s="138" t="n"/>
+      <c r="E69" s="138" t="n"/>
+      <c r="F69" s="138" t="n"/>
+      <c r="G69" s="138" t="n"/>
+      <c r="H69" s="139" t="n"/>
     </row>
     <row r="70" ht="24" customHeight="1" s="76">
       <c r="B70" s="11" t="inlineStr">
@@ -3185,6 +3195,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="76">
       <c r="A3" s="36" t="inlineStr">
         <is>
@@ -3192,6 +3203,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="76">
       <c r="A5" s="65" t="inlineStr">
         <is>
@@ -3326,6 +3338,8 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
     <row r="13" ht="24" customHeight="1" s="76">
       <c r="A13" s="65" t="inlineStr">
         <is>
@@ -3382,6 +3396,8 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
+    <row r="22"/>
     <row r="23" ht="24" customHeight="1" s="76">
       <c r="A23" s="65" t="inlineStr">
         <is>
@@ -3661,6 +3677,8 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
+    <row r="41"/>
     <row r="42" ht="24" customHeight="1" s="76">
       <c r="A42" s="65" t="inlineStr">
         <is>
@@ -89305,6 +89323,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="20.25" customHeight="1" s="76">
       <c r="A5" s="31" t="inlineStr">
         <is>
@@ -89336,6 +89355,7 @@
         <v/>
       </c>
     </row>
+    <row r="8"/>
     <row r="9" ht="34.65" customHeight="1" s="76">
       <c r="A9" s="39" t="inlineStr">
         <is>
@@ -89592,6 +89612,7 @@
         <v/>
       </c>
     </row>
+    <row r="18"/>
     <row r="19" ht="20.25" customHeight="1" s="76">
       <c r="A19" s="101" t="inlineStr">
         <is>
@@ -89599,6 +89620,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="28" customHeight="1" s="76">
       <c r="A21" s="82" t="inlineStr">
         <is>
@@ -89612,6 +89634,7 @@
       </c>
       <c r="D21" s="114" t="n"/>
     </row>
+    <row r="22"/>
     <row r="23" ht="24" customHeight="1" s="76">
       <c r="A23" s="45" t="inlineStr">
         <is>
@@ -89715,6 +89738,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="76">
       <c r="A5" s="49" t="inlineStr">
         <is>
@@ -89758,6 +89782,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10" ht="24" customHeight="1" s="76">
       <c r="A10" s="49" t="inlineStr">
         <is>
@@ -90176,6 +90201,8 @@
         <v>0.5</v>
       </c>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22" ht="24" customHeight="1" s="76">
       <c r="A22" s="49" t="inlineStr">
         <is>
@@ -90291,6 +90318,8 @@
       <c r="L26" s="71" t="n"/>
       <c r="M26" s="72" t="n"/>
     </row>
+    <row r="27"/>
+    <row r="28"/>
     <row r="29" ht="24" customHeight="1" s="76">
       <c r="A29" s="49" t="inlineStr">
         <is>
@@ -90901,6 +90930,7 @@
         </is>
       </c>
     </row>
+    <row r="39"/>
     <row r="40" ht="28" customHeight="1" s="76">
       <c r="A40" s="77" t="inlineStr">
         <is>
@@ -90971,6 +91001,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="20.25" customHeight="1" s="76">
       <c r="A5" s="57" t="inlineStr">
         <is>
@@ -91449,6 +91480,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="129" t="inlineStr">
         <is>
@@ -91459,10 +91491,20 @@
     <row r="6" ht="36" customHeight="1" s="76">
       <c r="A6" s="130" t="inlineStr">
         <is>
-          <t>Oui, pour 5 groupes sur 8, dont le paracétamol qui représente la moitié des ventes. Non pour l'asthme (R03) et l'ibuprofène (M01AE) ; gain trop faible pour l'aspirine (N02BA).</t>
-        </is>
-      </c>
-    </row>
+          <t>Oui, pour 5 groupes sur 8, dont le paracétamol qui représente la moitié des ventes. Non pour : Anti-inflammatoires type ibuprofène (M01AE), Asthme et BPCO (R03). Gain trop faible pour : Aspirine et dérivés (N02BA).</t>
+        </is>
+      </c>
+      <c r="B6" s="138" t="n"/>
+      <c r="C6" s="138" t="n"/>
+      <c r="D6" s="138" t="n"/>
+      <c r="E6" s="138" t="n"/>
+      <c r="F6" s="138" t="n"/>
+      <c r="G6" s="138" t="n"/>
+      <c r="H6" s="138" t="n"/>
+      <c r="I6" s="138" t="n"/>
+      <c r="J6" s="139" t="n"/>
+    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="129" t="inlineStr">
         <is>
@@ -91476,6 +91518,15 @@
           <t>1. On se replace chaque mois de janvier 2018 à septembre 2019 (21 mois) et on prévoit le mois suivant avec uniquement les ventes connues à ce moment-là. Puis on compare au vrai chiffre.</t>
         </is>
       </c>
+      <c r="B9" s="138" t="n"/>
+      <c r="C9" s="138" t="n"/>
+      <c r="D9" s="138" t="n"/>
+      <c r="E9" s="138" t="n"/>
+      <c r="F9" s="138" t="n"/>
+      <c r="G9" s="138" t="n"/>
+      <c r="H9" s="138" t="n"/>
+      <c r="I9" s="138" t="n"/>
+      <c r="J9" s="139" t="n"/>
     </row>
     <row r="10" ht="32" customHeight="1" s="76">
       <c r="A10" s="122" t="inlineStr">
@@ -91483,6 +91534,15 @@
           <t>2. Deux prévisions « naïves », que n'importe qui ferait sans nous : le mois prochain = le mois dernier ; le mois prochain = le même mois l'an dernier.</t>
         </is>
       </c>
+      <c r="B10" s="138" t="n"/>
+      <c r="C10" s="138" t="n"/>
+      <c r="D10" s="138" t="n"/>
+      <c r="E10" s="138" t="n"/>
+      <c r="F10" s="138" t="n"/>
+      <c r="G10" s="138" t="n"/>
+      <c r="H10" s="138" t="n"/>
+      <c r="I10" s="138" t="n"/>
+      <c r="J10" s="139" t="n"/>
     </row>
     <row r="11" ht="32" customHeight="1" s="76">
       <c r="A11" s="122" t="inlineStr">
@@ -91490,6 +91550,15 @@
           <t>3. Deux méthodes à nous : la moyenne des 3 derniers mois ; le niveau des 12 derniers mois corrigé de l'effet de saison du mois (« Saison x niveau »).</t>
         </is>
       </c>
+      <c r="B11" s="138" t="n"/>
+      <c r="C11" s="138" t="n"/>
+      <c r="D11" s="138" t="n"/>
+      <c r="E11" s="138" t="n"/>
+      <c r="F11" s="138" t="n"/>
+      <c r="G11" s="138" t="n"/>
+      <c r="H11" s="138" t="n"/>
+      <c r="I11" s="138" t="n"/>
+      <c r="J11" s="139" t="n"/>
     </row>
     <row r="12" ht="32" customHeight="1" s="76">
       <c r="A12" s="122" t="inlineStr">
@@ -91497,7 +91566,17 @@
           <t>4. Un groupe est jugé prévisible si notre meilleure méthode fait au moins 2 points d'erreur de moins que la meilleure naïve. En dessous, la différence peut être due au hasard.</t>
         </is>
       </c>
-    </row>
+      <c r="B12" s="138" t="n"/>
+      <c r="C12" s="138" t="n"/>
+      <c r="D12" s="138" t="n"/>
+      <c r="E12" s="138" t="n"/>
+      <c r="F12" s="138" t="n"/>
+      <c r="G12" s="138" t="n"/>
+      <c r="H12" s="138" t="n"/>
+      <c r="I12" s="138" t="n"/>
+      <c r="J12" s="139" t="n"/>
+    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="129" t="inlineStr">
         <is>
@@ -91861,6 +91940,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="129" t="inlineStr">
         <is>
@@ -91881,17 +91961,17 @@
       </c>
       <c r="C26" s="111" t="inlineStr">
         <is>
-          <t>Prévision oct. 2019</t>
+          <t>Prévision 10/2019</t>
         </is>
       </c>
       <c r="D26" s="111" t="inlineStr">
         <is>
-          <t>Réel sept. 2019</t>
+          <t>Réel 09/2019</t>
         </is>
       </c>
       <c r="E26" s="111" t="inlineStr">
         <is>
-          <t>Réel oct. 2018</t>
+          <t>Réel 10/2018</t>
         </is>
       </c>
       <c r="F26" s="111" t="inlineStr">
@@ -91929,10 +92009,10 @@
           <t>Saison x niveau (erreur moyenne 7.5 % sur 21 mois)</t>
         </is>
       </c>
-      <c r="G27" s="121" t="n"/>
-      <c r="H27" s="121" t="n"/>
-      <c r="I27" s="121" t="n"/>
-      <c r="J27" s="121" t="n"/>
+      <c r="G27" s="138" t="n"/>
+      <c r="H27" s="138" t="n"/>
+      <c r="I27" s="138" t="n"/>
+      <c r="J27" s="139" t="n"/>
     </row>
     <row r="28" ht="30" customHeight="1" s="76">
       <c r="A28" s="122" t="inlineStr">
@@ -91961,10 +92041,10 @@
           <t>Aucune méthode ne bat la prévision naïve : se fier au calendrier des saisons</t>
         </is>
       </c>
-      <c r="G28" s="121" t="n"/>
-      <c r="H28" s="121" t="n"/>
-      <c r="I28" s="121" t="n"/>
-      <c r="J28" s="121" t="n"/>
+      <c r="G28" s="138" t="n"/>
+      <c r="H28" s="138" t="n"/>
+      <c r="I28" s="138" t="n"/>
+      <c r="J28" s="139" t="n"/>
     </row>
     <row r="29" ht="30" customHeight="1" s="76">
       <c r="A29" s="122" t="inlineStr">
@@ -91993,10 +92073,10 @@
           <t>Aucune méthode ne bat la prévision naïve : se fier au calendrier des saisons</t>
         </is>
       </c>
-      <c r="G29" s="121" t="n"/>
-      <c r="H29" s="121" t="n"/>
-      <c r="I29" s="121" t="n"/>
-      <c r="J29" s="121" t="n"/>
+      <c r="G29" s="138" t="n"/>
+      <c r="H29" s="138" t="n"/>
+      <c r="I29" s="138" t="n"/>
+      <c r="J29" s="139" t="n"/>
     </row>
     <row r="30" ht="30" customHeight="1" s="76">
       <c r="A30" s="122" t="inlineStr">
@@ -92023,10 +92103,10 @@
           <t>Saison x niveau (erreur moyenne 13.0 % sur 21 mois)</t>
         </is>
       </c>
-      <c r="G30" s="121" t="n"/>
-      <c r="H30" s="121" t="n"/>
-      <c r="I30" s="121" t="n"/>
-      <c r="J30" s="121" t="n"/>
+      <c r="G30" s="138" t="n"/>
+      <c r="H30" s="138" t="n"/>
+      <c r="I30" s="138" t="n"/>
+      <c r="J30" s="139" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1" s="76">
       <c r="A31" s="122" t="inlineStr">
@@ -92053,10 +92133,10 @@
           <t>Moyenne 3 derniers mois (erreur moyenne 11.5 % sur 21 mois)</t>
         </is>
       </c>
-      <c r="G31" s="121" t="n"/>
-      <c r="H31" s="121" t="n"/>
-      <c r="I31" s="121" t="n"/>
-      <c r="J31" s="121" t="n"/>
+      <c r="G31" s="138" t="n"/>
+      <c r="H31" s="138" t="n"/>
+      <c r="I31" s="138" t="n"/>
+      <c r="J31" s="139" t="n"/>
     </row>
     <row r="32" ht="30" customHeight="1" s="76">
       <c r="A32" s="122" t="inlineStr">
@@ -92083,10 +92163,10 @@
           <t>Moyenne 3 derniers mois (erreur moyenne 33.8 % sur 21 mois)</t>
         </is>
       </c>
-      <c r="G32" s="121" t="n"/>
-      <c r="H32" s="121" t="n"/>
-      <c r="I32" s="121" t="n"/>
-      <c r="J32" s="121" t="n"/>
+      <c r="G32" s="138" t="n"/>
+      <c r="H32" s="138" t="n"/>
+      <c r="I32" s="138" t="n"/>
+      <c r="J32" s="139" t="n"/>
     </row>
     <row r="33" ht="30" customHeight="1" s="76">
       <c r="A33" s="122" t="inlineStr">
@@ -92115,10 +92195,10 @@
           <t>Aucune méthode ne bat la prévision naïve : se fier au calendrier des saisons</t>
         </is>
       </c>
-      <c r="G33" s="121" t="n"/>
-      <c r="H33" s="121" t="n"/>
-      <c r="I33" s="121" t="n"/>
-      <c r="J33" s="121" t="n"/>
+      <c r="G33" s="138" t="n"/>
+      <c r="H33" s="138" t="n"/>
+      <c r="I33" s="138" t="n"/>
+      <c r="J33" s="139" t="n"/>
     </row>
     <row r="34" ht="30" customHeight="1" s="76">
       <c r="A34" s="122" t="inlineStr">
@@ -92145,15 +92225,16 @@
           <t>Saison x niveau (erreur moyenne 19.0 % sur 21 mois)</t>
         </is>
       </c>
-      <c r="G34" s="121" t="n"/>
-      <c r="H34" s="121" t="n"/>
-      <c r="I34" s="121" t="n"/>
-      <c r="J34" s="121" t="n"/>
-    </row>
+      <c r="G34" s="138" t="n"/>
+      <c r="H34" s="138" t="n"/>
+      <c r="I34" s="138" t="n"/>
+      <c r="J34" s="139" t="n"/>
+    </row>
+    <row r="35"/>
     <row r="36" ht="32" customHeight="1" s="76">
       <c r="A36" s="127" t="inlineStr">
         <is>
-          <t>Octobre 2019 ne peut pas servir à vérifier la prévision : l'export s'arrête le 8 octobre. Ces chiffres sont produits par le script prevision.py, à relancer à chaque nouvel export.</t>
+          <t>Mise à jour automatique par classeur.ipynb avec l'export du 08/10/2019. Octobre 2019 ne peut pas encore servir à vérifier la prévision : il n'est pas terminé dans l'export.</t>
         </is>
       </c>
     </row>
@@ -92210,6 +92291,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="76">
       <c r="A3" s="36" t="inlineStr">
         <is>
@@ -92217,6 +92299,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="20.25" customHeight="1" s="76">
       <c r="A5" s="60" t="inlineStr">
         <is>
@@ -92435,6 +92518,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="20.25" customHeight="1" s="76">
       <c r="A5" s="61" t="inlineStr">
         <is>
@@ -92802,6 +92886,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="28" customHeight="1" s="76">
       <c r="A3" s="36" t="inlineStr">
         <is>
@@ -92809,6 +92894,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="20.25" customHeight="1" s="76">
       <c r="A5" s="62" t="inlineStr">
         <is>
@@ -93119,6 +93205,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5" ht="24" customHeight="1" s="76">
       <c r="A5" s="63" t="inlineStr">
         <is>
@@ -93188,7 +93275,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="34.65" customHeight="1" s="76">
+    <row r="7" ht="20.25" customHeight="1" s="76">
       <c r="A7" s="70" t="inlineStr">
         <is>
           <t>M01AB</t>
@@ -93230,7 +93317,7 @@
         <v>211.1</v>
       </c>
     </row>
-    <row r="8" ht="34.65" customHeight="1" s="76">
+    <row r="8" ht="20.25" customHeight="1" s="76">
       <c r="A8" s="70" t="inlineStr">
         <is>
           <t>M01AE</t>
@@ -95256,7 +95343,7 @@
         </is>
       </c>
     </row>
-    <row r="82">
+    <row r="82" ht="20.25" customHeight="1" s="76">
       <c r="A82" s="70" t="n">
         <v>2014</v>
       </c>
@@ -95288,7 +95375,7 @@
         <v>2.24</v>
       </c>
     </row>
-    <row r="83">
+    <row r="83" ht="20.25" customHeight="1" s="76">
       <c r="A83" s="70" t="n">
         <v>2015</v>
       </c>
@@ -95320,7 +95407,7 @@
         <v>2.74</v>
       </c>
     </row>
-    <row r="84">
+    <row r="84" ht="20.25" customHeight="1" s="76">
       <c r="A84" s="70" t="n">
         <v>2016</v>
       </c>
@@ -95352,7 +95439,7 @@
         <v>2.94</v>
       </c>
     </row>
-    <row r="85">
+    <row r="85" ht="20.25" customHeight="1" s="76">
       <c r="A85" s="70" t="n">
         <v>2017</v>
       </c>
@@ -95384,7 +95471,7 @@
         <v>2.67</v>
       </c>
     </row>
-    <row r="86">
+    <row r="86" ht="20.25" customHeight="1" s="76">
       <c r="A86" s="70" t="n">
         <v>2018</v>
       </c>
@@ -95416,7 +95503,7 @@
         <v>3.32</v>
       </c>
     </row>
-    <row r="87">
+    <row r="87" ht="20.25" customHeight="1" s="76">
       <c r="A87" s="70" t="n">
         <v>2019</v>
       </c>

</xml_diff>

<commit_message>
Python : interface avec résultats et catégories de médicaments
</commit_message>
<xml_diff>
--- a/excel/Pharma_Analyse.xlsx
+++ b/excel/Pharma_Analyse.xlsx
@@ -15,8 +15,9 @@
     <sheet name="Médicaments" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Méthode" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Statistiques" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="État des données" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Données" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Catégories" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="État des données" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Données" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="DateMin">MIN(Données!$A$2:$A$2107)</definedName>
@@ -3171,6 +3172,529 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="FFD5DCF7"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E37"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" style="76" min="1" max="1"/>
+    <col width="44" customWidth="1" style="76" min="2" max="2"/>
+    <col width="26" customWidth="1" style="76" min="3" max="3"/>
+    <col width="16" customWidth="1" style="76" min="4" max="4"/>
+    <col width="16" customWidth="1" style="76" min="5" max="5"/>
+    <col width="16" customWidth="1" style="76" min="6" max="6"/>
+    <col width="16" customWidth="1" style="76" min="7" max="7"/>
+    <col width="16" customWidth="1" style="76" min="8" max="8"/>
+    <col width="16" customWidth="1" style="76" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="109" t="inlineStr">
+        <is>
+          <t>Catégories de médicaments</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="89" t="inlineStr">
+        <is>
+          <t>Groupes rangés par catégorie grâce à leur code ATC. Les quantités de médicaments différents sont additionnées : à utiliser pour suivre une catégorie dans le temps, pas pour comparer deux catégories.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="36" t="inlineStr">
+        <is>
+          <t>◀ Accueil</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="63" t="inlineStr">
+        <is>
+          <t>CORRESPONDANCE CODE ATC → CATÉGORIE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="64" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B6" s="64" t="inlineStr">
+        <is>
+          <t>Sous-groupe ATC</t>
+        </is>
+      </c>
+      <c r="C6" s="64" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+      <c r="D6" s="64" t="inlineStr">
+        <is>
+          <t>Nouveau ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="70" t="inlineStr">
+        <is>
+          <t>M01AB</t>
+        </is>
+      </c>
+      <c r="B7" s="70" t="inlineStr">
+        <is>
+          <t>Dérivés de l'acide acétique (diclofénac)</t>
+        </is>
+      </c>
+      <c r="C7" s="70" t="inlineStr">
+        <is>
+          <t>Douleur et inflammation</t>
+        </is>
+      </c>
+      <c r="D7" s="70" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="70" t="inlineStr">
+        <is>
+          <t>M01AE</t>
+        </is>
+      </c>
+      <c r="B8" s="70" t="inlineStr">
+        <is>
+          <t>Dérivés de l'acide propionique (ibuprofène)</t>
+        </is>
+      </c>
+      <c r="C8" s="70" t="inlineStr">
+        <is>
+          <t>Douleur et inflammation</t>
+        </is>
+      </c>
+      <c r="D8" s="70" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="70" t="inlineStr">
+        <is>
+          <t>N02BA</t>
+        </is>
+      </c>
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>Acide salicylique et dérivés (aspirine)</t>
+        </is>
+      </c>
+      <c r="C9" s="70" t="inlineStr">
+        <is>
+          <t>Douleur et inflammation</t>
+        </is>
+      </c>
+      <c r="D9" s="70" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="70" t="inlineStr">
+        <is>
+          <t>N02BE</t>
+        </is>
+      </c>
+      <c r="B10" s="70" t="inlineStr">
+        <is>
+          <t>Anilides (paracétamol)</t>
+        </is>
+      </c>
+      <c r="C10" s="70" t="inlineStr">
+        <is>
+          <t>Douleur et inflammation</t>
+        </is>
+      </c>
+      <c r="D10" s="70" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="70" t="inlineStr">
+        <is>
+          <t>N05B</t>
+        </is>
+      </c>
+      <c r="B11" s="70" t="inlineStr">
+        <is>
+          <t>Anxiolytiques</t>
+        </is>
+      </c>
+      <c r="C11" s="70" t="inlineStr">
+        <is>
+          <t>Anxiété et sommeil</t>
+        </is>
+      </c>
+      <c r="D11" s="70" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="70" t="inlineStr">
+        <is>
+          <t>N05C</t>
+        </is>
+      </c>
+      <c r="B12" s="70" t="inlineStr">
+        <is>
+          <t>Hypnotiques et sédatifs</t>
+        </is>
+      </c>
+      <c r="C12" s="70" t="inlineStr">
+        <is>
+          <t>Anxiété et sommeil</t>
+        </is>
+      </c>
+      <c r="D12" s="70" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="70" t="inlineStr">
+        <is>
+          <t>R03</t>
+        </is>
+      </c>
+      <c r="B13" s="70" t="inlineStr">
+        <is>
+          <t>Médicaments de l'asthme et de la BPCO</t>
+        </is>
+      </c>
+      <c r="C13" s="70" t="inlineStr">
+        <is>
+          <t>Respiratoire</t>
+        </is>
+      </c>
+      <c r="D13" s="70" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="70" t="inlineStr">
+        <is>
+          <t>R06</t>
+        </is>
+      </c>
+      <c r="B14" s="70" t="inlineStr">
+        <is>
+          <t>Antihistaminiques</t>
+        </is>
+      </c>
+      <c r="C14" s="70" t="inlineStr">
+        <is>
+          <t>Allergies</t>
+        </is>
+      </c>
+      <c r="D14" s="70" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="63" t="inlineStr">
+        <is>
+          <t>VENTES MOYENNES PAR MOIS, PAR CATÉGORIE ET PAR ANNÉE</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="64" t="inlineStr">
+        <is>
+          <t>Année</t>
+        </is>
+      </c>
+      <c r="B18" s="64" t="inlineStr">
+        <is>
+          <t>Allergies</t>
+        </is>
+      </c>
+      <c r="C18" s="64" t="inlineStr">
+        <is>
+          <t>Anxiété et sommeil</t>
+        </is>
+      </c>
+      <c r="D18" s="64" t="inlineStr">
+        <is>
+          <t>Douleur et inflammation</t>
+        </is>
+      </c>
+      <c r="E18" s="64" t="inlineStr">
+        <is>
+          <t>Respiratoire</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="70" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B19" s="70" t="n">
+        <v>69.3</v>
+      </c>
+      <c r="C19" s="70" t="n">
+        <v>385.9</v>
+      </c>
+      <c r="D19" s="70" t="n">
+        <v>1128</v>
+      </c>
+      <c r="E19" s="70" t="n">
+        <v>103.7</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="70" t="n">
+        <v>2015</v>
+      </c>
+      <c r="B20" s="70" t="n">
+        <v>83.40000000000001</v>
+      </c>
+      <c r="C20" s="70" t="n">
+        <v>262.2</v>
+      </c>
+      <c r="D20" s="70" t="n">
+        <v>1428.1</v>
+      </c>
+      <c r="E20" s="70" t="n">
+        <v>147.7</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="70" t="n">
+        <v>2016</v>
+      </c>
+      <c r="B21" s="70" t="n">
+        <v>89.7</v>
+      </c>
+      <c r="C21" s="70" t="n">
+        <v>280.9</v>
+      </c>
+      <c r="D21" s="70" t="n">
+        <v>1579.9</v>
+      </c>
+      <c r="E21" s="70" t="n">
+        <v>179.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="70" t="n">
+        <v>2017</v>
+      </c>
+      <c r="B22" s="70" t="n">
+        <v>81.09999999999999</v>
+      </c>
+      <c r="C22" s="70" t="n">
+        <v>210.2</v>
+      </c>
+      <c r="D22" s="70" t="n">
+        <v>1164.1</v>
+      </c>
+      <c r="E22" s="70" t="n">
+        <v>158.2</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="70" t="n">
+        <v>2018</v>
+      </c>
+      <c r="B23" s="70" t="n">
+        <v>101</v>
+      </c>
+      <c r="C23" s="70" t="n">
+        <v>295.3</v>
+      </c>
+      <c r="D23" s="70" t="n">
+        <v>1324.4</v>
+      </c>
+      <c r="E23" s="70" t="n">
+        <v>225.5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="70" t="n">
+        <v>2019</v>
+      </c>
+      <c r="B24" s="70" t="n">
+        <v>119.5</v>
+      </c>
+      <c r="C24" s="70" t="n">
+        <v>283.4</v>
+      </c>
+      <c r="D24" s="70" t="n">
+        <v>1259</v>
+      </c>
+      <c r="E24" s="70" t="n">
+        <v>213.6</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="63" t="inlineStr">
+        <is>
+          <t>ÉVOLUTION SUR UN AN (12 DERNIERS MOIS COMPLETS CONTRE LES 12 PRÉCÉDENTS)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="64" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+      <c r="B28" s="64" t="inlineStr">
+        <is>
+          <t>12 derniers mois</t>
+        </is>
+      </c>
+      <c r="C28" s="64" t="inlineStr">
+        <is>
+          <t>12 mois précédents</t>
+        </is>
+      </c>
+      <c r="D28" s="64" t="inlineStr">
+        <is>
+          <t>Évolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="70" t="inlineStr">
+        <is>
+          <t>Allergies</t>
+        </is>
+      </c>
+      <c r="B29" s="70" t="n">
+        <v>1261.3</v>
+      </c>
+      <c r="C29" s="70" t="n">
+        <v>1174.6</v>
+      </c>
+      <c r="D29" s="70" t="inlineStr">
+        <is>
+          <t>+7 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="70" t="inlineStr">
+        <is>
+          <t>Anxiété et sommeil</t>
+        </is>
+      </c>
+      <c r="B30" s="70" t="n">
+        <v>3439.8</v>
+      </c>
+      <c r="C30" s="70" t="n">
+        <v>3349</v>
+      </c>
+      <c r="D30" s="70" t="inlineStr">
+        <is>
+          <t>+3 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="70" t="inlineStr">
+        <is>
+          <t>Douleur et inflammation</t>
+        </is>
+      </c>
+      <c r="B31" s="70" t="n">
+        <v>15928.4</v>
+      </c>
+      <c r="C31" s="70" t="n">
+        <v>15598.7</v>
+      </c>
+      <c r="D31" s="70" t="inlineStr">
+        <is>
+          <t>+2 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="70" t="inlineStr">
+        <is>
+          <t>Respiratoire</t>
+        </is>
+      </c>
+      <c r="B32" s="70" t="n">
+        <v>2962.7</v>
+      </c>
+      <c r="C32" s="70" t="n">
+        <v>2323.2</v>
+      </c>
+      <c r="D32" s="70" t="inlineStr">
+        <is>
+          <t>+28 %</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="63" t="inlineStr">
+        <is>
+          <t>NOUVEAUX MÉDICAMENTS DÉTECTÉS DANS CET EXPORT</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="64" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B36" s="64" t="inlineStr">
+        <is>
+          <t>Catégorie</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="70" t="inlineStr">
+        <is>
+          <t>Aucun</t>
+        </is>
+      </c>
+      <c r="B37" s="70" t="inlineStr">
+        <is>
+          <t>L'export contient les mêmes 8 groupes qu'au départ.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
     <tabColor rgb="FFE3E3C3"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -4963,7 +5487,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FFE0E0E0"/>
@@ -91515,7 +92039,7 @@
     <row r="9" ht="32" customHeight="1" s="76">
       <c r="A9" s="122" t="inlineStr">
         <is>
-          <t>1. On se replace chaque mois de janvier 2018 à septembre 2019 (21 mois) et on prévoit le mois suivant avec uniquement les ventes connues à ce moment-là. Puis on compare au vrai chiffre.</t>
+          <t>1. On fait comme si on était dans le passé : avec les seules ventes connues jusqu'à décembre 2017, on prévoit janvier 2018, puis on compare au vrai chiffre. On répète chaque mois jusqu'à septembre 2019 : 21 prévisions testées.</t>
         </is>
       </c>
       <c r="B9" s="138" t="n"/>

</xml_diff>